<commit_message>
fix bug for inconsistant name for the thermal zone Messe
</commit_message>
<xml_diff>
--- a/data/tek_data/TEK_Teilenergiekennwerte.xlsx
+++ b/data/tek_data/TEK_Teilenergiekennwerte.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" codeName="DieseArbeitsmappe" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <workbookPr filterPrivacy="1" codeName="DieseArbeitsmappe"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94D6CBF-8F76-485A-B853-9B05E9AD3463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="4"/>
+    <workbookView xWindow="1515" yWindow="3000" windowWidth="21600" windowHeight="11280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sehr hoch" sheetId="1" r:id="rId1"/>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="60">
   <si>
     <t>Einzelbüro</t>
   </si>
@@ -196,11 +197,14 @@
   <si>
     <t>Küche – Vorbereitung, Lager</t>
   </si>
+  <si>
+    <t>Messe / Kongress</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -517,7 +521,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2095,7 +2099,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3670,7 +3674,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5245,7 +5249,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6821,7 +6825,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7771,7 +7775,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
inconsistant name for Messe
</commit_message>
<xml_diff>
--- a/data/tek_data/TEK_Teilenergiekennwerte.xlsx
+++ b/data/tek_data/TEK_Teilenergiekennwerte.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr filterPrivacy="1" codeName="DieseArbeitsmappe"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94D6CBF-8F76-485A-B853-9B05E9AD3463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA513723-966D-4E5C-8EEA-4D447AD75423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="3000" windowWidth="21600" windowHeight="11280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="2655" windowWidth="21600" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sehr hoch" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="59">
   <si>
     <t>Einzelbüro</t>
   </si>
@@ -109,9 +109,6 @@
   </si>
   <si>
     <t>Bühne (Theater und Veranstaltungsbauten)</t>
-  </si>
-  <si>
-    <t>Messe/Kongress</t>
   </si>
   <si>
     <t>Ausstellungsräume und Museum mit konservatorischen Anforderungen</t>
@@ -541,37 +538,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>47</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -614,7 +611,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -789,7 +786,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -1034,7 +1031,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -1069,7 +1066,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -1334,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>
@@ -1474,7 +1471,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -1509,7 +1506,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
         <v>1</v>
@@ -1544,7 +1541,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>1</v>
@@ -1579,7 +1576,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>1</v>
@@ -1614,7 +1611,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>1</v>
@@ -1649,7 +1646,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>1</v>
@@ -1684,7 +1681,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34">
         <v>222</v>
@@ -1716,7 +1713,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35">
         <v>740.4</v>
@@ -1853,7 +1850,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
         <v>1</v>
@@ -1923,7 +1920,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>1</v>
@@ -1958,7 +1955,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
@@ -1993,7 +1990,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -2063,7 +2060,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>
@@ -2116,37 +2113,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>47</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -2189,7 +2186,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -2364,7 +2361,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -2609,7 +2606,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -2644,7 +2641,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -2909,7 +2906,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>
@@ -3049,7 +3046,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -3084,7 +3081,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
         <v>1</v>
@@ -3119,7 +3116,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>1</v>
@@ -3154,7 +3151,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>1</v>
@@ -3189,7 +3186,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>1</v>
@@ -3224,7 +3221,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>1</v>
@@ -3259,7 +3256,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34">
         <v>71.7</v>
@@ -3291,7 +3288,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35">
         <v>223.1</v>
@@ -3428,7 +3425,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
         <v>1</v>
@@ -3498,7 +3495,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>1</v>
@@ -3533,7 +3530,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
@@ -3568,7 +3565,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -3638,7 +3635,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>
@@ -3691,37 +3688,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>47</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -3764,7 +3761,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -3939,7 +3936,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -4184,7 +4181,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -4219,7 +4216,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -4484,7 +4481,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>
@@ -4624,7 +4621,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -4659,7 +4656,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
         <v>1</v>
@@ -4694,7 +4691,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>1</v>
@@ -4729,7 +4726,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>1</v>
@@ -4764,7 +4761,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>1</v>
@@ -4799,7 +4796,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>1</v>
@@ -4834,7 +4831,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34">
         <v>45.5</v>
@@ -4866,7 +4863,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35">
         <v>144.9</v>
@@ -5003,7 +5000,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
         <v>1</v>
@@ -5073,7 +5070,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>1</v>
@@ -5108,7 +5105,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
@@ -5143,7 +5140,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -5213,7 +5210,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>
@@ -5267,37 +5264,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>47</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -5340,7 +5337,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -5515,7 +5512,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -5760,7 +5757,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -5795,7 +5792,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -6060,7 +6057,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>
@@ -6200,7 +6197,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -6235,7 +6232,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
         <v>1</v>
@@ -6270,7 +6267,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>1</v>
@@ -6305,7 +6302,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>1</v>
@@ -6340,7 +6337,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>1</v>
@@ -6375,7 +6372,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>1</v>
@@ -6410,7 +6407,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34">
         <v>23.1</v>
@@ -6442,7 +6439,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35">
         <v>64.3</v>
@@ -6579,7 +6576,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
         <v>1</v>
@@ -6649,7 +6646,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>1</v>
@@ -6684,7 +6681,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
@@ -6719,7 +6716,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -6789,7 +6786,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>
@@ -6842,37 +6839,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>47</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -6915,7 +6912,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -7090,7 +7087,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -7335,7 +7332,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -7370,7 +7367,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -7635,7 +7632,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>
@@ -7775,7 +7772,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -7810,7 +7807,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
         <v>1</v>
@@ -7845,7 +7842,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>1</v>
@@ -7880,7 +7877,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>1</v>
@@ -7915,7 +7912,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>1</v>
@@ -7950,7 +7947,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>1</v>
@@ -7985,7 +7982,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34">
         <v>10.3</v>
@@ -8017,7 +8014,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35">
         <v>26.7</v>
@@ -8154,7 +8151,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
         <v>1</v>
@@ -8224,7 +8221,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>1</v>
@@ -8259,7 +8256,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
@@ -8294,7 +8291,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -8364,7 +8361,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>

</xml_diff>